<commit_message>
Se agrega paso de ModifyColumnValues, se agregan pasos a la data.
</commit_message>
<xml_diff>
--- a/data/database/metric_dimensions.xlsx
+++ b/data/database/metric_dimensions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,6 +560,14 @@
         <v>13</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>